<commit_message>
docs: adiciona anotacoes e planilha pratica sobre a funcao offset.
</commit_message>
<xml_diff>
--- a/01_Excel_PowerQuery/Excel Impressionador - Hashtag/planilhas/funcao_match_e_index.xlsx
+++ b/01_Excel_PowerQuery/Excel Impressionador - Hashtag/planilhas/funcao_match_e_index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaof\Desktop\Excel Impressionador 2021\Módulo 8 - Funções Mercado de Trabalho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF5C0BCD-C684-43BC-AB69-E0B0B9A28E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83D4BC66-901F-4CFA-854B-228C6647A3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{90D394A7-0334-4363-9DA1-420D95C76B52}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="4" activeTab="4" xr2:uid="{90D394A7-0334-4363-9DA1-420D95C76B52}"/>
   </bookViews>
   <sheets>
     <sheet name="CORRESP" sheetId="2" r:id="rId1"/>
@@ -209,10 +209,10 @@
     <t>Coluna</t>
   </si>
   <si>
-    <t>CORRESP</t>
+    <t>MATCH</t>
   </si>
   <si>
-    <t>ÍNDICE</t>
+    <t>INDEX</t>
   </si>
   <si>
     <t>PROCURA</t>
@@ -222,9 +222,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -315,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -356,6 +357,10 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5185,8 +5190,8 @@
         <v>10</v>
       </c>
       <c r="G3" s="11" t="str" cm="1">
-        <f t="array" ref="G3">INDEX(A2:A16,G2)</f>
-        <v>Produto 5</v>
+        <f t="array" ref="G3">INDEX(B2:B16,G2)</f>
+        <v>H1935</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -5220,7 +5225,7 @@
         <v>44</v>
       </c>
       <c r="G5" s="9">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -5240,7 +5245,7 @@
         <v>45</v>
       </c>
       <c r="G6" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -5256,9 +5261,9 @@
       <c r="D7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="11" t="str" cm="1">
+      <c r="G7" s="11" cm="1">
         <f t="array" ref="G7">INDEX(A2:D16,G5,G6)</f>
-        <v>Alpha</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -7179,7 +7184,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7236,16 +7241,16 @@
         <v>0</v>
       </c>
       <c r="G4" s="5">
-        <f>MATCH($G$1,$B$2:$B$16,0)</f>
-        <v>5</v>
+        <f>MATCH(G1,B2:B16,0)</f>
+        <v>8</v>
       </c>
       <c r="H4" s="1" t="str" cm="1">
-        <f t="array" ref="H4">INDEX($A$2:$A$16,G4)</f>
-        <v>Produto 5</v>
+        <f t="array" ref="H4">INDEX(A2:D16,G4,1)</f>
+        <v>Produto 8</v>
       </c>
       <c r="I4" s="1" t="str">
-        <f>INDEX(A:A,MATCH($G$1,B:B,0))</f>
-        <v>Produto 5</v>
+        <f>INDEX($A:$D,MATCH($G$1,$B:$B,0),MATCH($F4,$A$1:$D$1,0))</f>
+        <v>Produto 8</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -7265,16 +7270,16 @@
         <v>2</v>
       </c>
       <c r="G5" s="5">
-        <f t="shared" ref="G5:G6" si="0">MATCH($G$1,$B$2:$B$16,0)</f>
-        <v>5</v>
-      </c>
-      <c r="H5" s="6" cm="1">
-        <f t="array" ref="H5">INDEX($C$2:$C$16,G5)</f>
-        <v>6228</v>
-      </c>
-      <c r="I5" s="6">
-        <f>INDEX(C:C,MATCH($G$1,B:B,0))</f>
-        <v>6228</v>
+        <f>MATCH(G1,B2:B16,0)</f>
+        <v>8</v>
+      </c>
+      <c r="H5" s="18" cm="1">
+        <f t="array" ref="H5">INDEX(A2:D16,G5,3)</f>
+        <v>8222</v>
+      </c>
+      <c r="I5" s="17">
+        <f t="shared" ref="I5:I6" si="0">INDEX($A:$D,MATCH($G$1,$B:$B,0),MATCH($F5,$A$1:$D$1,0))</f>
+        <v>8222</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -7294,16 +7299,16 @@
         <v>3</v>
       </c>
       <c r="G6" s="5">
+        <f>MATCH(G1,B2:B16,0)</f>
+        <v>8</v>
+      </c>
+      <c r="H6" s="1" t="str" cm="1">
+        <f t="array" ref="H6">INDEX(A2:D16,G6,4)</f>
+        <v>Beta</v>
+      </c>
+      <c r="I6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H6" s="1" t="str" cm="1">
-        <f t="array" ref="H6">INDEX($D$2:$D$16,G6)</f>
-        <v>Alpha</v>
-      </c>
-      <c r="I6" s="1" t="str">
-        <f>INDEX(D:D,MATCH($G$1,B:B,0))</f>
-        <v>Alpha</v>
+        <v>Beta</v>
       </c>
     </row>
     <row r="7" spans="1:9">

</xml_diff>